<commit_message>
EDC v1.2: Mexico labor and machine rate estimates, "press size" naming
- Labor $3.50/hr (x 0.5 operators); machine bands $31 / $42 / $56 / $77, marked as Mexico estimates
- "Press used" is now "Press size" in the workbook and web tool
- Web tool uses a new saved-state key so earlier saved inputs pick up the new defaults
- Parity check still 1024/1024

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ensu1vNHvKEJQ5TzFuE1wc
</commit_message>
<xml_diff>
--- a/EDC_Cost_Estimator_v1.2.xlsx
+++ b/EDC_Cost_Estimator_v1.2.xlsx
@@ -295,7 +295,7 @@
     </comment>
     <comment ref="B21" authorId="0" shapeId="0">
       <text>
-        <t>Placeholder for Durango, Mexico. Enter your plant's loaded operator rate.</t>
+        <t>Mexico estimate. Enter your plant's loaded operator rate.</t>
       </text>
     </comment>
     <comment ref="B22" authorId="0" shapeId="0">
@@ -310,7 +310,7 @@
     </comment>
     <comment ref="A27" authorId="0" shapeId="0">
       <text>
-        <t>Blank = rate from the Assumptions band of the press used. Machine only, no labor.</t>
+        <t>Blank = rate from the Assumptions band of the press size. Machine only, no labor.</t>
       </text>
     </comment>
     <comment ref="A28" authorId="0" shapeId="0">
@@ -355,7 +355,7 @@
     </comment>
     <comment ref="C47" authorId="0" shapeId="0">
       <text>
-        <t>North American placeholders. Replace with Durango machine rates (machine only; labor is entered separately).</t>
+        <t>Mexico estimates (machine only). Replace with Durango machine rates (machine only; labor is entered separately).</t>
       </text>
     </comment>
   </commentList>
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="B21" s="16" t="n">
-        <v>6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="22">
@@ -992,7 +992,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Press used (US t)</t>
+          <t>Press size (US t)</t>
         </is>
       </c>
       <c r="B26" s="10" t="n"/>
@@ -1300,7 +1300,7 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>Press used (US t)</t>
+          <t>Press size (US t)</t>
         </is>
       </c>
       <c r="B45" s="19">
@@ -1939,7 +1939,7 @@
         <v>300</v>
       </c>
       <c r="C47" s="16" t="n">
-        <v>45</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48">
@@ -1952,7 +1952,7 @@
         <v>500</v>
       </c>
       <c r="C48" s="16" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49">
@@ -1965,7 +1965,7 @@
         <v>800</v>
       </c>
       <c r="C49" s="16" t="n">
-        <v>80</v>
+        <v>56</v>
       </c>
     </row>
     <row r="50">
@@ -1980,7 +1980,7 @@
         </is>
       </c>
       <c r="C50" s="16" t="n">
-        <v>110</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52">
@@ -2007,7 +2007,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>Press used = your press tons on the Estimator if entered, else the rule of thumb. Machine rate comes from the band of the press used unless overridden.</t>
+          <t>Press size = your press tons on the Estimator if entered, else the rule of thumb. Machine rate comes from the band of the press size unless overridden.</t>
         </is>
       </c>
     </row>
@@ -2966,7 +2966,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Press used (US t)</t>
+          <t>Press size (US t)</t>
         </is>
       </c>
       <c r="B44" s="12">
@@ -3364,7 +3364,7 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>Press used (US t)</t>
+          <t>Press size (US t)</t>
         </is>
       </c>
       <c r="B62" s="12">
@@ -3762,7 +3762,7 @@
     <row r="80">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>Press used (US t)</t>
+          <t>Press size (US t)</t>
         </is>
       </c>
       <c r="B80" s="12">

</xml_diff>